<commit_message>
feat: enhance site with 4+ myths & faqs per page, page-tailored CTAs, gold branding, header/footer fixes, and updated SEO audits
</commit_message>
<xml_diff>
--- a/scripts/MBA_Wizards_SEO_Audit.xlsx
+++ b/scripts/MBA_Wizards_SEO_Audit.xlsx
@@ -760,22 +760,22 @@
         <v>https://www.mbawizards.co.in/blogs</v>
       </c>
       <c r="D6" t="str">
-        <v>⚠️ Desc Too Long, ⚠️ No Keywords</v>
+        <v>❌ No Meta Title, ❌ No Meta Description, ⚠️ No Keywords</v>
       </c>
       <c r="E6" t="str">
-        <v>75%</v>
+        <v>63%</v>
       </c>
       <c r="F6" t="str">
-        <v>MBA Preparation Blog &amp; Admissions Insights | MBA Wizards</v>
+        <v/>
       </c>
       <c r="G6">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="H6" t="str">
-        <v>Explore 100+ expert guides on GMAT Focus Edition, GRE strategies, CAT preparation, top MBA interview questions, application essays, and success stories by IIT Roorkee alumni.</v>
+        <v/>
       </c>
       <c r="I6">
-        <v>174</v>
+        <v>0</v>
       </c>
       <c r="J6" t="str">
         <v/>
@@ -4824,22 +4824,22 @@
         <v>https://www.mbawizards.co.in/blogs</v>
       </c>
       <c r="D6" t="str">
-        <v>⚠️ Desc Too Long, ⚠️ No Keywords</v>
+        <v>❌ No Meta Title, ❌ No Meta Description, ⚠️ No Keywords</v>
       </c>
       <c r="E6" t="str">
-        <v>75%</v>
+        <v>63%</v>
       </c>
       <c r="F6" t="str">
-        <v>MBA Preparation Blog &amp; Admissions Insights | MBA Wizards</v>
+        <v/>
       </c>
       <c r="G6">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="H6" t="str">
-        <v>Explore 100+ expert guides on GMAT Focus Edition, GRE strategies, CAT preparation, top MBA interview questions, application essays, and success stories by IIT Roorkee alumni.</v>
+        <v/>
       </c>
       <c r="I6">
-        <v>174</v>
+        <v>0</v>
       </c>
       <c r="J6" t="str">
         <v/>
@@ -8696,10 +8696,10 @@
         <v>https://www.mbawizards.co.in/blogs</v>
       </c>
       <c r="D6" t="str">
-        <v>75%</v>
+        <v>63%</v>
       </c>
       <c r="E6" t="str">
-        <v>⚠️ Desc Too Long, ⚠️ No Keywords</v>
+        <v>❌ No Meta Title, ❌ No Meta Description, ⚠️ No Keywords</v>
       </c>
       <c r="F6" t="str">
         <v>MBA &amp; GMAT Blog | Expert Tips, Guides &amp; Interview Prep | MBA Wizards</v>

</xml_diff>